<commit_message>
fixed issues from review
</commit_message>
<xml_diff>
--- a/rules/CORE-000362/negative/01/data/unit-test-coreid-CG0037-negative 1.xlsx
+++ b/rules/CORE-000362/negative/01/data/unit-test-coreid-CG0037-negative 1.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -62,9 +62,18 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -78,6 +87,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -107,7 +128,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -115,6 +136,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -500,7 +523,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F17"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -556,10 +579,10 @@
         <v>5</v>
       </c>
       <c r="E3" s="4" t="str">
-        <v>AEBDSYCD</v>
-      </c>
-      <c r="F3" s="4">
-        <v>111</v>
+        <v>AEDECOD</v>
+      </c>
+      <c r="F3" s="4" t="str">
+        <v>Pneumonia</v>
       </c>
     </row>
     <row r="4">
@@ -576,15 +599,15 @@
         <v>5</v>
       </c>
       <c r="E4" s="4" t="str">
-        <v>AESOCCD</v>
+        <v>AEBDSYCD</v>
       </c>
       <c r="F4" s="4">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" s="4" t="str">
         <v>ae.xpt</v>
@@ -593,13 +616,13 @@
         <v>Record</v>
       </c>
       <c r="D5" s="4">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E5" s="4" t="str">
-        <v>AETERM</v>
-      </c>
-      <c r="F5" s="4" t="str">
-        <v>URINARY TRACT INFECTION</v>
+        <v>AESOCCD</v>
+      </c>
+      <c r="F5" s="4">
+        <v>112</v>
       </c>
     </row>
     <row r="6">
@@ -616,10 +639,10 @@
         <v>6</v>
       </c>
       <c r="E6" s="4" t="str">
-        <v>AEBDSYCD</v>
-      </c>
-      <c r="F6" s="4">
-        <v>110</v>
+        <v>AETERM</v>
+      </c>
+      <c r="F6" s="4" t="str">
+        <v>URINARY TRACT INFECTION</v>
       </c>
     </row>
     <row r="7">
@@ -636,15 +659,15 @@
         <v>6</v>
       </c>
       <c r="E7" s="4" t="str">
-        <v>AESOCCD</v>
-      </c>
-      <c r="F7" s="4">
-        <v>112</v>
+        <v>AEDECOD</v>
+      </c>
+      <c r="F7" s="4" t="str">
+        <v>Urinary tract infection</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B8" s="4" t="str">
         <v>ae.xpt</v>
@@ -653,18 +676,18 @@
         <v>Record</v>
       </c>
       <c r="D8" s="4">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E8" s="4" t="str">
-        <v>AETERM</v>
-      </c>
-      <c r="F8" s="4" t="str">
-        <v>UPSET STOMACH</v>
+        <v>AEBDSYCD</v>
+      </c>
+      <c r="F8" s="4">
+        <v>110</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B9" s="4" t="str">
         <v>ae.xpt</v>
@@ -673,13 +696,13 @@
         <v>Record</v>
       </c>
       <c r="D9" s="4">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E9" s="4" t="str">
-        <v>AEBDSYCD</v>
+        <v>AESOCCD</v>
       </c>
       <c r="F9" s="4">
-        <v>123</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10">
@@ -696,15 +719,15 @@
         <v>7</v>
       </c>
       <c r="E10" s="4" t="str">
-        <v>AESOCCD</v>
-      </c>
-      <c r="F10" s="4">
-        <v>124</v>
+        <v>AETERM</v>
+      </c>
+      <c r="F10" s="4" t="str">
+        <v>UPSET STOMACH</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B11" s="4" t="str">
         <v>ae.xpt</v>
@@ -713,18 +736,18 @@
         <v>Record</v>
       </c>
       <c r="D11" s="4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E11" s="4" t="str">
-        <v>AETERM</v>
+        <v>AEDECOD</v>
       </c>
       <c r="F11" s="4" t="str">
-        <v>BACK PAIN</v>
+        <v>Abdominal discomfort</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B12" s="4" t="str">
         <v>ae.xpt</v>
@@ -733,18 +756,18 @@
         <v>Record</v>
       </c>
       <c r="D12" s="4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E12" s="4" t="str">
         <v>AEBDSYCD</v>
       </c>
-      <c r="F12" s="4" t="str">
-        <v/>
+      <c r="F12" s="4">
+        <v>123</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B13" s="4" t="str">
         <v>ae.xpt</v>
@@ -753,18 +776,98 @@
         <v>Record</v>
       </c>
       <c r="D13" s="4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E13" s="4" t="str">
         <v>AESOCCD</v>
       </c>
       <c r="F13" s="4">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4">
+        <v>4</v>
+      </c>
+      <c r="B14" s="4" t="str">
+        <v>ae.xpt</v>
+      </c>
+      <c r="C14" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D14" s="4">
+        <v>8</v>
+      </c>
+      <c r="E14" s="4" t="str">
+        <v>AETERM</v>
+      </c>
+      <c r="F14" s="4" t="str">
+        <v>BACK PAIN</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4">
+        <v>4</v>
+      </c>
+      <c r="B15" s="4" t="str">
+        <v>ae.xpt</v>
+      </c>
+      <c r="C15" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D15" s="4">
+        <v>8</v>
+      </c>
+      <c r="E15" s="4" t="str">
+        <v>AEDECOD</v>
+      </c>
+      <c r="F15" s="4" t="str">
+        <v>Back pain</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4">
+        <v>4</v>
+      </c>
+      <c r="B16" s="4" t="str">
+        <v>ae.xpt</v>
+      </c>
+      <c r="C16" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D16" s="4">
+        <v>8</v>
+      </c>
+      <c r="E16" s="4" t="str">
+        <v>AEBDSYCD</v>
+      </c>
+      <c r="F16" s="4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4">
+        <v>4</v>
+      </c>
+      <c r="B17" s="4" t="str">
+        <v>ae.xpt</v>
+      </c>
+      <c r="C17" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D17" s="4">
+        <v>8</v>
+      </c>
+      <c r="E17" s="4" t="str">
+        <v>AESOCCD</v>
+      </c>
+      <c r="F17" s="4">
         <v>111</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F17"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -863,257 +966,257 @@
       <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="6" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Sponsor-Defined Identifier</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Reported Term for the Adverse Event</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Lowest Level Term</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="6" t="str">
         <v>Lowest Level Term Code</v>
       </c>
-      <c r="I2" s="5" t="str">
+      <c r="I2" s="6" t="str">
         <v>Dictionary-Derived Term</v>
       </c>
-      <c r="J2" s="5" t="str">
+      <c r="J2" s="6" t="str">
         <v>Preferred Term Code</v>
       </c>
-      <c r="K2" s="5" t="str">
+      <c r="K2" s="6" t="str">
         <v>High Level Term</v>
       </c>
-      <c r="L2" s="5" t="str">
+      <c r="L2" s="6" t="str">
         <v>High Level Term Code</v>
       </c>
-      <c r="M2" s="5" t="str">
+      <c r="M2" s="6" t="str">
         <v>High Level Group Term</v>
       </c>
-      <c r="N2" s="5" t="str">
+      <c r="N2" s="6" t="str">
         <v>High Level Group Term Code</v>
       </c>
-      <c r="O2" s="5" t="str">
+      <c r="O2" s="6" t="str">
         <v>Subcategory for Adverse Event</v>
       </c>
-      <c r="P2" s="5" t="str">
+      <c r="P2" s="6" t="str">
         <v>Body System or Organ Class</v>
       </c>
-      <c r="Q2" s="5" t="str">
+      <c r="Q2" s="6" t="str">
         <v>Body System or Organ Class Code</v>
       </c>
-      <c r="R2" s="5" t="str">
+      <c r="R2" s="6" t="str">
         <v>Primary System Organ Class</v>
       </c>
-      <c r="S2" s="5" t="str">
+      <c r="S2" s="6" t="str">
         <v>Primary System Organ Class Code</v>
       </c>
-      <c r="T2" s="5" t="str">
+      <c r="T2" s="6" t="str">
         <v>Severity/Intensity</v>
       </c>
-      <c r="U2" s="5" t="str">
+      <c r="U2" s="6" t="str">
         <v>Serious Event</v>
       </c>
-      <c r="V2" s="5" t="str">
+      <c r="V2" s="6" t="str">
         <v>Action Taken with Study Treatment</v>
       </c>
-      <c r="W2" s="5" t="str">
+      <c r="W2" s="6" t="str">
         <v>Causality</v>
       </c>
-      <c r="X2" s="5" t="str">
+      <c r="X2" s="6" t="str">
         <v>Outcome of Adverse Event</v>
       </c>
-      <c r="Y2" s="5" t="str">
+      <c r="Y2" s="6" t="str">
         <v>Requires or Prolongs Hospitalization</v>
       </c>
-      <c r="Z2" s="5" t="str">
+      <c r="Z2" s="6" t="str">
         <v>Start Date/Time of Adverse Event</v>
       </c>
-      <c r="AA2" s="5" t="str">
+      <c r="AA2" s="6" t="str">
         <v>End Date/Time of Adverse Event</v>
       </c>
-      <c r="AB2" s="5" t="str">
+      <c r="AB2" s="6" t="str">
         <v>Study Day of Start of Adverse Event</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="5" t="str">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="5" t="str">
+      <c r="E3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="I3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="5" t="str">
+      <c r="I3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="K3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="L3" s="5" t="str">
+      <c r="K3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="L3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="M3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="N3" s="5" t="str">
+      <c r="M3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="N3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="O3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="P3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Q3" s="5" t="str">
+      <c r="O3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="P3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Q3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="R3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="S3" s="5" t="str">
+      <c r="R3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="S3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="T3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="U3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="V3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="W3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="X3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Y3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Z3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AA3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AB3" s="5" t="str">
+      <c r="T3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="U3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="V3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="W3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="X3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Y3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Z3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AA3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AB3" s="6" t="str">
         <v>Num</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
+      <c r="A4" s="6">
         <v>10</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="6">
         <v>2</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="6">
         <v>14</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="6">
         <v>8</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="6">
         <v>4</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="6">
         <v>38</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="6">
         <v>38</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="6">
         <v>8</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="6">
         <v>38</v>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="6">
         <v>8</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="6">
         <v>65</v>
       </c>
-      <c r="L4" s="5">
+      <c r="L4" s="6">
         <v>8</v>
       </c>
-      <c r="M4" s="5">
+      <c r="M4" s="6">
         <v>55</v>
       </c>
-      <c r="N4" s="5">
+      <c r="N4" s="6">
         <v>8</v>
       </c>
-      <c r="O4" s="5">
+      <c r="O4" s="6">
         <v>200</v>
       </c>
-      <c r="P4" s="5">
+      <c r="P4" s="6">
         <v>52</v>
       </c>
-      <c r="Q4" s="5">
+      <c r="Q4" s="6">
         <v>8</v>
       </c>
-      <c r="R4" s="5">
+      <c r="R4" s="6">
         <v>52</v>
       </c>
-      <c r="S4" s="5">
+      <c r="S4" s="6">
         <v>8</v>
       </c>
-      <c r="T4" s="5">
+      <c r="T4" s="6">
         <v>8</v>
       </c>
-      <c r="U4" s="5">
+      <c r="U4" s="6">
         <v>1</v>
       </c>
-      <c r="V4" s="5">
+      <c r="V4" s="6">
         <v>1</v>
       </c>
-      <c r="W4" s="5">
+      <c r="W4" s="6">
         <v>1</v>
       </c>
-      <c r="X4" s="5">
+      <c r="X4" s="6">
         <v>26</v>
       </c>
-      <c r="Y4" s="5">
+      <c r="Y4" s="6">
         <v>1</v>
       </c>
-      <c r="Z4" s="5">
+      <c r="Z4" s="6">
         <v>10</v>
       </c>
-      <c r="AA4" s="5">
+      <c r="AA4" s="6">
         <v>1</v>
       </c>
-      <c r="AB4" s="5">
+      <c r="AB4" s="6">
         <v>8</v>
       </c>
     </row>
@@ -1133,7 +1236,7 @@
       <c r="E5" s="4">
         <v>1586</v>
       </c>
-      <c r="F5" s="6" t="str">
+      <c r="F5" s="7" t="str">
         <v>PNEUMONIA</v>
       </c>
       <c r="G5" s="4" t="str">
@@ -1142,7 +1245,7 @@
       <c r="H5" s="4">
         <v>10035664</v>
       </c>
-      <c r="I5" s="4" t="str">
+      <c r="I5" s="8" t="str">
         <v>Pneumonia</v>
       </c>
       <c r="J5" s="4">
@@ -1166,13 +1269,13 @@
       <c r="P5" s="4" t="str">
         <v>Infections and infestations</v>
       </c>
-      <c r="Q5" s="6">
+      <c r="Q5" s="8">
         <v>111</v>
       </c>
       <c r="R5" s="4" t="str">
         <v>Cardiac disorders</v>
       </c>
-      <c r="S5" s="6">
+      <c r="S5" s="8">
         <v>112</v>
       </c>
       <c r="T5" s="4" t="str">
@@ -1219,7 +1322,7 @@
       <c r="E6" s="4">
         <v>1594</v>
       </c>
-      <c r="F6" s="6" t="str">
+      <c r="F6" s="8" t="str">
         <v>URINARY TRACT INFECTION</v>
       </c>
       <c r="G6" s="4" t="str">
@@ -1228,7 +1331,7 @@
       <c r="H6" s="4">
         <v>10046571</v>
       </c>
-      <c r="I6" s="4" t="str">
+      <c r="I6" s="8" t="str">
         <v>Urinary tract infection</v>
       </c>
       <c r="J6" s="4">
@@ -1252,13 +1355,13 @@
       <c r="P6" s="4" t="str">
         <v>Cardiac disorders</v>
       </c>
-      <c r="Q6" s="6">
+      <c r="Q6" s="8">
         <v>110</v>
       </c>
       <c r="R6" s="4" t="str">
         <v>CARDIAC disorders</v>
       </c>
-      <c r="S6" s="6">
+      <c r="S6" s="8">
         <v>112</v>
       </c>
       <c r="T6" s="4" t="str">
@@ -1305,7 +1408,7 @@
       <c r="E7" s="4">
         <v>1603</v>
       </c>
-      <c r="F7" s="6" t="str">
+      <c r="F7" s="8" t="str">
         <v>UPSET STOMACH</v>
       </c>
       <c r="G7" s="4" t="str">
@@ -1314,7 +1417,7 @@
       <c r="H7" s="4">
         <v>10046318</v>
       </c>
-      <c r="I7" s="4" t="str">
+      <c r="I7" s="8" t="str">
         <v>Abdominal discomfort</v>
       </c>
       <c r="J7" s="4">
@@ -1338,13 +1441,13 @@
       <c r="P7" s="4" t="str">
         <v>Musculoskeletal and connective tissue disorders</v>
       </c>
-      <c r="Q7" s="6">
+      <c r="Q7" s="8">
         <v>123</v>
       </c>
       <c r="R7" s="4" t="str">
         <v>Gastrointestinal disorders</v>
       </c>
-      <c r="S7" s="6">
+      <c r="S7" s="8">
         <v>124</v>
       </c>
       <c r="T7" s="4" t="str">
@@ -1391,7 +1494,7 @@
       <c r="E8" s="4">
         <v>1615</v>
       </c>
-      <c r="F8" s="6" t="str">
+      <c r="F8" s="8" t="str">
         <v>BACK PAIN</v>
       </c>
       <c r="G8" s="4" t="str">
@@ -1400,7 +1503,7 @@
       <c r="H8" s="4">
         <v>10003988</v>
       </c>
-      <c r="I8" s="4" t="str">
+      <c r="I8" s="8" t="str">
         <v>Back pain</v>
       </c>
       <c r="J8" s="4">
@@ -1424,13 +1527,13 @@
       <c r="P8" s="4" t="str">
         <v>Musculoskeletal and connective TISSUE disorders</v>
       </c>
-      <c r="Q8" s="6" t="str">
+      <c r="Q8" s="8" t="str">
         <v/>
       </c>
       <c r="R8" s="4" t="str">
         <v>Musculoskeletal and connective tissue disorders</v>
       </c>
-      <c r="S8" s="6">
+      <c r="S8" s="8">
         <v>111</v>
       </c>
       <c r="T8" s="4" t="str">

</xml_diff>